<commit_message>
Add real download URLs to data sources sheet + raw README
Data_Sources_and_Gaps.xlsx now leads with a 'Download Links' sheet: every layer
with a clickable City Open Data / agency URL, dataset ID, status, and how to
download. Mirrored the core links in src/data/raw/README.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Data_Sources_and_Gaps.xlsx
+++ b/docs/Data_Sources_and_Gaps.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Download Links" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Needed From City" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Status Key" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -39,9 +39,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="005C6670"/>
-      <sz val="9"/>
+      <color rgb="001155CC"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="8">
@@ -63,22 +63,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FBE3DF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECEAE3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DDE7F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCEFC7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FBE3DF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E4E2DA"/>
       </patternFill>
     </fill>
   </fills>
@@ -119,6 +119,9 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -131,7 +134,6 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -497,39 +499,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Layer</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>What it governs / used for</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Agency</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Dataset ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Layer / Dataset</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Owner (Agency)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Feeds (rule)</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
@@ -537,320 +539,320 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Source / How obtained</t>
+          <t>How to download</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Download URL</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DS-034</t>
+          <t>Sidewalks (planimetric)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Subway Entrances &amp; Exits (2,120 pts citywide)</t>
+          <t>Where vending is physically allowed — the green areas</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>MTA / NY State</t>
+          <t>DCP</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>10 ft no-vend buffer (both vendor types)</t>
+          <t>vfx9-tbb6</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>In use (live)</t>
+          <t>Live</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>NY Open Data resource i9wp-a4ja — data.ny.gov (fetched 2026-06-04, bundled)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Real data, all five boroughs. Drives the subway exclusion.</t>
+          <t>NYC Open Data — use the Export button (GeoJSON or Shapefile)</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>https://data.cityofnewyork.us/d/vfx9-tbb6</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Zoning Districts (C4/C5/C6)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Borough Boundaries</t>
+          <t>Commercial-zone exclusion for General Vendors</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>NYC DCP</t>
+          <t>DCP</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Determines which borough a point is in (food borough permits)</t>
+          <t>nyzd</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>In use (live)</t>
+          <t>Live</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>NYC Open Data resource gthc-hcne — data.cityofnewyork.us (fetched + simplified, bundled)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Real data; simplified for fast point-in-polygon.</t>
+          <t>DCP "BYTES of the Big Apple" — Shapefile (nyzd)</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nyc.gov/content/planning/pages/resources/datasets/gis-zoning-features</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Parks Properties</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Basemap (streets, labels)</t>
+          <t>Out of scope (parks use a separate DPR permit system)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>OpenStreetMap / OpenFreeMap</t>
+          <t>DPR</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Visual base layer</t>
+          <t>enfh-gkve</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>In use (live)</t>
+          <t>Live</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>OpenFreeMap Positron vector tiles (no key, no usage limits)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Open data; not a City source. Could swap to a City basemap later.</t>
+          <t>NYC Open Data — Export GeoJSON</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>https://data.cityofnewyork.us/d/enfh-gkve</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>§20-465(g)(1)</t>
+          <t>Subway Entrances &amp; Exits</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Midtown Core zone</t>
+          <t>10 ft no-vend buffer (both vendor types)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>DCWP (NYC Admin Code)</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Blue-license-only area (GV)</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Encoded from statute</t>
+          <t>i9wp-a4ja</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Boundary text in the Admin Code — encoded as an approximate polygon</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>No file needed; geometry is approximate, confirm exact lines.</t>
+          <t>NY State Open Data — Export CSV/GeoJSON</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>https://data.ny.gov/d/i9wp-a4ja</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>§20-465(g)(4)</t>
+          <t>Fire Hydrants</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Downtown Flushing zone</t>
+          <t>10 ft no-vend buffer (distance pending legal confirm)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>DCWP (NYC Admin Code)</t>
+          <t>NYCDEP</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Standard-GV exclusion</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Encoded from statute</t>
+          <t>6pui-xhxz</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Boundary text in the Admin Code — encoded as an approximate polygon</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>No file needed; approximate.</t>
+          <t>NYC Open Data — Export CSV (has lat/long)</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>https://data.cityofnewyork.us/d/6pui-xhxz</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>§20-465(g)(5)</t>
+          <t>Borough Boundaries</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Dyker Heights zone (seasonal)</t>
+          <t>Borough-specific permit geography</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>DCWP (NYC Admin Code)</t>
+          <t>DCP</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Holiday-hours GV restriction</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Encoded from statute</t>
+          <t>gthc-hcne</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Boundary text in the Admin Code — encoded as an approximate polygon</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>No file needed; approximate.</t>
+          <t>NYC Open Data — Export GeoJSON</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>https://data.cityofnewyork.us/d/gthc-hcne</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>DS-012</t>
+          <t>Basemap tiles</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Zoning — C4 / C5 / C6 districts</t>
+          <t>Map background</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>DCP</t>
+          <t>OpenStreetMap / OpenFreeMap</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Commercial-zone exclusion (GV)</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Illustrative placeholder</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Live</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Map-type dataset; not exportable as queryable GeoJSON. Using sample polygons.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>NEED the licensed GIS Zoning Features export to be accurate.</t>
+          <t>Open vector tiles, no API key</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>https://openfreemap.org</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>DS-032</t>
+          <t>DCWP General Vendor street restrictions</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Parks Properties</t>
+          <t>AUTHORITATIVE permitted/prohibited GV streets (the existing DCWP map)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>DPR</t>
+          <t>DCWP</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Out-of-scope mask (parks)</t>
+          <t>DS-007</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Illustrative placeholder</t>
+          <t>Needed</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Using sample polygons (Central Park, Prospect Park)</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>NEED DPR parks polygons for full coverage.</t>
+          <t>Public ArcGIS map (linked from DSNY page); WRITTEN LICENSE required for production use</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nyc.gov/site/dsny/what-we-do/cleaning/street-vending-enforcement.page</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>DS-005</t>
+          <t>DOHMH Restricted Streets (Mobile Food)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Green Cart precincts</t>
+          <t>Food time/day street restrictions (the #1 food input)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -860,34 +862,34 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Green Cart authorized geography</t>
+          <t>DS-001</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Illustrative placeholder</t>
+          <t>Needed</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Using one sample precinct polygon</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>NEED DOHMH Green Cart precinct polygons (or a precinct list to convert).</t>
+          <t>Public map online; GIS layer with hours/days via DOHMH agency request</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>https://a816-dohbesp.nyc.gov/IndicatorPublic/mobilefoodvending</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>DS-001</t>
+          <t>Green Cart precincts</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>DOHMH Restricted Streets (hours/days)</t>
+          <t>Green Cart authorized geography (police-precinct based)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -897,665 +899,418 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Food time/day restrictions (the #1 food input)</t>
+          <t>DS-005</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Illustrative placeholder</t>
+          <t>Needed</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Using one sample restricted street</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>NEED DOHMH GIS layer with per-segment hours/days (or PDF to geocode).</t>
+          <t>Precinct list/polygons via DOHMH agency request (Local Law 9 of 2008)</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nyc.gov/site/doh/business/food-operators/mobile-and-temporary-food-vendors.page</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>DS-036</t>
+          <t>Building Footprints</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Fire hydrants</t>
+          <t>20 ft building/store-entrance buffer</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>FDNY / DEP</t>
+          <t>DCP</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Hydrant no-vend buffer</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Illustrative placeholder</t>
+          <t>5zhs-2jue</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Map-type dataset, ~100k points — too large to bundle. Using sample point.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>NEED a hydrant layer via a spatial service. Stay-away DISTANCE also unverified.</t>
+          <t>NYC Open Data — Export GeoJSON</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>https://data.cityofnewyork.us/d/5zhs-2jue</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Bicycle Routes / Lanes</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Scaffolding / sidewalk sheds</t>
+          <t>No vending in bike lanes</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>DOB</t>
+          <t>DOT</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Obstruction advisory</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Illustrative placeholder</t>
+          <t>mzxg-pwib</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Using sample point</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>NEED DOB active sidewalk-shed permits (updates frequently).</t>
+          <t>NYC Open Data — Export GeoJSON</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>https://data.cityofnewyork.us/d/mzxg-pwib</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>DS-007</t>
+          <t>Bus Stop Shelters</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>General Vendor street restrictions</t>
+          <t>5 ft GV buffer</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>DCWP</t>
+          <t>DOT</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Authoritative GV permitted/prohibited streets</t>
+          <t>t4f2-8md7</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Missing — needed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Public ArcGIS map exists but not ingested</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>NEED a written license to use in production. This IS the existing DCWP map; required to replace it.</t>
+          <t>NYC Open Data — Export GeoJSON</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>https://data.cityofnewyork.us/d/t4f2-8md7</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>DS-041</t>
+          <t>Pedestrian Plazas (polygon)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Sidewalk polygons (planimetrics)</t>
+          <t>Out of scope (concession-only)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>DCP / DOT</t>
+          <t>DOT</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Confines vending to actual sidewalks; green "allowed" areas</t>
+          <t>k5k6-6jex</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Missing — needed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Not exposed as a client-usable service; full layer is very large</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>NEED the sidewalk shapefile + a spatial backend. Blocker for the green allowed-area map.</t>
+          <t>NYC Open Data — Export GeoJSON</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>https://data.cityofnewyork.us/d/k5k6-6jex</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>DS-040</t>
+          <t>Parking Regulation Locations &amp; Signs</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Sidewalk widths</t>
+          <t>No-standing zones / metered-parking rule</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>DOT / community</t>
+          <t>DOT</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>12 ft clearance rule</t>
+          <t>nfid-uabd</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Missing — needed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Not yet sourced</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>NEED widths per segment (or derive from DS-041).</t>
+          <t>NYC Open Data — Export</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>https://data.cityofnewyork.us/d/nfid-uabd</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Street Centerline (CSCL)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Base join key; crosswalk &amp; corner buffers</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>DCP</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
           <t>DS-013</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Street Centerline (CSCL)</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>DCP</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Base join key for every street-level rule</t>
-        </is>
-      </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Missing — needed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Public, refreshes daily</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>NEED to ingest as the production base layer.</t>
+          <t>NYC Open Data — search "NYC Street Centerline (CSCL)"</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>https://opendata.cityofnewyork.us/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DS-014</t>
+          <t>Sidewalk widths</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>LION street network</t>
+          <t>12 ft clearance rule</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>DCP</t>
+          <t>DOT / community</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Partial-block "from X to Y" segments</t>
+          <t>DS-040</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Missing — needed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>NEED for sub-segment encoding of restricted streets.</t>
+          <t>Derive from the sidewalk polygons (above) or community data</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>https://data.cityofnewyork.us/d/vfx9-tbb6</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>DS-015</t>
+          <t>Scaffolding / sidewalk sheds</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Building Footprints</t>
+          <t>Obstruction advisory</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>DCP</t>
+          <t>DOB</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>20 ft building-entrance buffer</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Missing — needed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>NEED (entrances approximated from footprint edge).</t>
+          <t>NYC Open Data — search "DOB NOW: Build – Approved Permits" (filter Sidewalk Shed)</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>https://opendata.cityofnewyork.us/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>DS-026</t>
+          <t>Newsstands</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Pedestrian Plazas</t>
+          <t>5 ft GV buffer</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>DOT</t>
+          <t>DCWP</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Out-of-scope mask (plazas)</t>
+          <t>DS-—</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Missing — needed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>NEED plaza polygons.</t>
+          <t>DCWP licensed-premises / NYC Open Data — search "Newsstand"</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>https://opendata.cityofnewyork.us/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>DS-027</t>
+          <t>Sidewalk cafés</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Bus Stop Shelters</t>
+          <t>20 ft buffer</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>DOT</t>
+          <t>DCWP</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>5 ft GV buffer</t>
+          <t>DS-—</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Missing — needed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>NEED shelter locations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>DS-028</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>No-Standing signs</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>DOT</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Hospital no-standing zones</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Missing — needed</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>NEED sign data (paired with hospital locations).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>DS-029</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Curb cuts / driveways</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>DOT</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>10 ft driveway buffer</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>Missing — needed</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>No clean citywide layer found</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>GAP — may need OSM/footprint approximation; flag to vendors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>DS-031</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Crosswalks (derived)</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>DOT / from CSCL</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>10 ft MFV crosswalk buffer</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>Missing — needed</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Derive from CSCL</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>NEED CSCL first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>DS-035</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>MTA Bus Stops</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>MTA</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>No vending within a bus stop</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>Missing — needed</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>NEED stop boundaries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>DS-003</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Restricted Area Permit zones</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>DOHMH</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Separate food SKU (high-traffic zones)</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>Missing — needed</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Confirm scope</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>NEED to confirm if in scope + boundaries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>DS-023</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>ECB / OATH citation records</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>DSNY</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Evaluation metrics (not map logic)</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Missing — needed</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Gated</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>NEED for measuring impact (Deliverable metrics).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>C-1</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>World Trade Center zone</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>DCWP / DOHMH (Admin Code)</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Hard prohibition + MFV street exceptions</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>Blocked (legal)</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Conflict C-1: docs say Barclay St; 2023 DCWP guide says Vesey St</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>NOT a file — needs SBS Legal to confirm the controlling boundary before encoding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Compiled 2026-06-04 for the Street Vendor Site Selection Tool (prototype). Statuses reflect what the live app uses. "Missing — needed" + "Illustrative placeholder" rows are the asks for the City.</t>
+          <t>NYC Open Data — search "Sidewalk Café"</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>https://opendata.cityofnewyork.us/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A30:G30"/>
-  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1566,44 +1321,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Dataset ID</t>
+          <t>Dataset / item</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Layer / Dataset</t>
+          <t>Agency</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Agency</t>
+          <t>Why we need it</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Why we need it</t>
+          <t>Ask / blocker</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Ask / blocker</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
@@ -1612,30 +1361,25 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DS-001</t>
+          <t>DS-007 — DCWP General Vendor street restrictions</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DOHMH Restricted Streets (GIS, hours/days)</t>
+          <t>DCWP</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>DOHMH</t>
+          <t>Authoritative legal streets; required to replace the DCWP map</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>The single most important food input; powers the time view</t>
+          <t>Execute the written license; confirm live-service vs. static export</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Request GIS export with per-segment hours/days</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1644,30 +1388,25 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DS-005</t>
+          <t>DS-001 — DOHMH Restricted Streets (GIS)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Green Cart precincts</t>
+          <t>DOHMH</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>DOHMH</t>
+          <t>The #1 food input; powers the time view</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Show Green Cart vendors their authorized area</t>
+          <t>Request GIS export with per-segment hours/days</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Request precinct polygons (or list to convert)</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1676,30 +1415,25 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>DS-007</t>
+          <t>DS-005 — Green Cart precincts</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>General Vendor street restrictions</t>
+          <t>DOHMH</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>DCWP</t>
+          <t>Where Green Cart vendors may operate</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Authoritative GV legal streets; required to replace the DCWP map</t>
+          <t>Request precinct polygons (or list to convert)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Execute written license; confirm consume-live-vs-static</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1708,350 +1442,106 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>DS-012</t>
+          <t>Buffers: building entrances, bike lanes, bus shelters, plazas, no-standing, crosswalks, bus stops</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>GIS Zoning Features (C4/C5/C6)</t>
+          <t>DCP / DOT / MTA</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>DCP</t>
+          <t>Distance-buffer prohibitions + out-of-scope masks</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Accurate commercial-zone exclusion for GV</t>
+          <t>Ingest the public layers (links on the first sheet); derive crosswalks from CSCL</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Licensed GIS export (not the map-only service)</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>DS-013</t>
+          <t>Fire-hydrant stay-away distance</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Street Centerline (CSCL)</t>
+          <t>SBS Legal / FDNY</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>DCP</t>
+          <t>Engine uses 10 ft but the code only confirms a no-contact rule</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Base join key for every street rule</t>
+          <t>Confirm the controlling distance</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Confirm ingest cadence (daily refresh)</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>DS-034</t>
+          <t>C-1 — WTC zone boundary</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Subway Entrances</t>
+          <t>SBS Legal / DCWP</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>Encode the WTC hard prohibition correctly</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Already in use — confirm we may use it in production</t>
+          <t>Confirm Barclay vs. Vesey St (§20-465(g)(2))</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Confirm license/currency of the Open Data version</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>P1 (have data)</t>
+          <t>P1 (legal)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>DS-041</t>
+          <t>C-6 — Tool vs. existing agency maps</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Sidewalk polygons (planimetrics)</t>
+          <t>SBS / DSNY</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>DCP / DOT</t>
+          <t>Decides whether this replaces / federates / links the agency maps</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Green "where you CAN vend" areas; confine vending to sidewalks</t>
+          <t>Confirm the intended relationship — gates the data architecture</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Provide shapefile + agree on a spatial backend/tiles</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>P1 (blocks green map)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>DS-040</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Sidewalk widths</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>DOT</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>12 ft clearance rule</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Provide widths or confirm derive from DS-041</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>DS-015 / 027 / 028 / 035 / 026 / 031 / 029</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Buffers: building entrances, bus shelters, no-standing, bus stops, plazas, crosswalks, driveways</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>DCP / DOT / MTA</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Distance-buffer prohibitions (§10 step 5) and out-of-scope masks</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Provide layers / confirm DOT-internal driveway data</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>DS-036</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Fire hydrants</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>FDNY / DEP</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Hydrant no-vend buffer</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Provide hydrant layer; CONFIRM the legal stay-away distance</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Active sidewalk-shed (scaffolding) permits</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>DOB</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Flag spots physically blocked by scaffolding</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Provide a feed (changes frequently)</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>DS-023</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>ECB / OATH citation records</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>DSNY</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Evaluation metrics for the pilot</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Provide aggregate citation data</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>C-1</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>WTC zone boundary</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>SBS Legal / DCWP</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Encode the WTC hard-prohibition correctly</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>CONFIRM Barclay vs Vesey St north border (§20-465(g)(2))</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>P1 (legal, not data)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>C-6</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Tool relationship to existing maps</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>SBS / DSNY</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Decides whether we replace / federate / link agency maps</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>CONFIRM the intended relationship — gates the data architecture</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>P1 (decision)</t>
         </is>
@@ -2071,11 +1561,11 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="86" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
@@ -2090,60 +1580,60 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>In use (live)</t>
+          <t>Live</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Real authoritative data is wired in and affects results.</t>
+          <t>Real City data is downloaded, processed, and wired into the app.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Encoded from statute</t>
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Statutory</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Geometry encoded from the Admin Code boundary text (approximate). No file required.</t>
+          <t>Zone geometry encoded from the Admin Code text (Midtown Core, Flushing, Dyker Heights) — no file needed.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Illustrative placeholder</t>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Illustrative</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Sample geometry standing in until the licensed/acquired dataset arrives.</t>
+          <t>Sample geometry in the app today; swap for the real download when obtained.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Missing — needed</t>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Needed</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Not yet integrated; the rule cannot fully work until the City provides the data.</t>
+          <t>Gated / agency data that governs where vendors operate — request or license required.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Blocked (legal)</t>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Needs a legal/policy decision, not just a file.</t>
+          <t>Public layer, not yet integrated; download link provided.</t>
         </is>
       </c>
     </row>

</xml_diff>